<commit_message>
v341: 7 more Process Control Tables read from their PDFs (F12, F19, F28 UFG3, F30 Stage 2, FCS0105, FCS0205, F72 Stage 2): control data on asset pages, control tags, Sources, Checks; off Ref Only. PDF reader: older headings, two-row column headings, template order for the sideways alarm columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KTEDhnU5tNU91Jmkwz9aQB
</commit_message>
<xml_diff>
--- a/sources/pct1410001.xlsx
+++ b/sources/pct1410001.xlsx
@@ -1012,85 +1012,37 @@
           <t>P_LL</t>
         </is>
       </c>
-      <c r="Q6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay ON (sec)</t>
-        </is>
-      </c>
-      <c r="R6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay OFF (sec)</t>
-        </is>
-      </c>
+      <c r="Q6" s="1" t="inlineStr"/>
+      <c r="R6" s="1" t="inlineStr"/>
       <c r="S6" s="1" t="inlineStr"/>
-      <c r="T6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay OFF (sec)</t>
-        </is>
-      </c>
-      <c r="U6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay OFF (sec)</t>
-        </is>
-      </c>
-      <c r="V6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay OFF (sec)</t>
-        </is>
-      </c>
-      <c r="W6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay OFF (sec)</t>
-        </is>
-      </c>
+      <c r="T6" s="1" t="inlineStr"/>
+      <c r="U6" s="1" t="inlineStr"/>
+      <c r="V6" s="1" t="inlineStr"/>
+      <c r="W6" s="1" t="inlineStr"/>
       <c r="X6" s="1" t="inlineStr"/>
       <c r="Y6" s="1" t="inlineStr">
         <is>
           <t>P_HH</t>
         </is>
       </c>
-      <c r="Z6" s="1" t="inlineStr">
-        <is>
-          <t>P_HH Delay ON (sec)</t>
-        </is>
-      </c>
-      <c r="AA6" s="1" t="inlineStr">
-        <is>
-          <t>P_HH Delay OFF (sec)</t>
-        </is>
-      </c>
+      <c r="Z6" s="1" t="inlineStr"/>
+      <c r="AA6" s="1" t="inlineStr"/>
       <c r="AB6" s="1" t="inlineStr">
         <is>
           <t>A_LL</t>
         </is>
       </c>
-      <c r="AC6" s="1" t="inlineStr">
-        <is>
-          <t>A_LL Delay (sec)</t>
-        </is>
-      </c>
+      <c r="AC6" s="1" t="inlineStr"/>
       <c r="AD6" s="1" t="inlineStr"/>
-      <c r="AE6" s="1" t="inlineStr">
-        <is>
-          <t>A_LL Delay (sec)</t>
-        </is>
-      </c>
-      <c r="AF6" s="1" t="inlineStr">
-        <is>
-          <t>A_LL Delay (sec)</t>
-        </is>
-      </c>
+      <c r="AE6" s="1" t="inlineStr"/>
+      <c r="AF6" s="1" t="inlineStr"/>
       <c r="AG6" s="1" t="inlineStr"/>
       <c r="AH6" s="1" t="inlineStr">
         <is>
           <t>A_HH</t>
         </is>
       </c>
-      <c r="AI6" s="1" t="inlineStr">
-        <is>
-          <t>A_HH Delay (sec)</t>
-        </is>
-      </c>
+      <c r="AI6" s="1" t="inlineStr"/>
       <c r="AJ6" s="1" t="inlineStr">
         <is>
           <t>Alarm Masking Conditions</t>
@@ -1121,11 +1073,7 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="AP6" s="1" t="inlineStr">
-        <is>
-          <t>A_HH Delay (sec)</t>
-        </is>
-      </c>
+      <c r="AP6" s="1" t="inlineStr"/>
       <c r="AQ6" s="1" t="inlineStr">
         <is>
           <t>Destination (Output) Tag</t>
@@ -13859,18 +13807,10 @@
           <t>P_LL</t>
         </is>
       </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay ON (sec)</t>
-        </is>
-      </c>
+      <c r="J6" s="1" t="inlineStr"/>
       <c r="K6" s="1" t="inlineStr"/>
       <c r="L6" s="1" t="inlineStr"/>
-      <c r="M6" s="1" t="inlineStr">
-        <is>
-          <t>P_LL Delay OFF (sec)</t>
-        </is>
-      </c>
+      <c r="M6" s="1" t="inlineStr"/>
       <c r="N6" s="1" t="inlineStr"/>
       <c r="O6" s="1" t="inlineStr"/>
       <c r="P6" s="1" t="inlineStr"/>
@@ -13880,11 +13820,7 @@
           <t>P_HH</t>
         </is>
       </c>
-      <c r="S6" s="1" t="inlineStr">
-        <is>
-          <t>P_HH Delay ON (sec)</t>
-        </is>
-      </c>
+      <c r="S6" s="1" t="inlineStr"/>
       <c r="T6" s="1" t="inlineStr"/>
       <c r="U6" s="1" t="inlineStr">
         <is>
@@ -13896,16 +13832,24 @@
           <t>A_LL Delay (sec)</t>
         </is>
       </c>
-      <c r="W6" s="1" t="inlineStr"/>
+      <c r="W6" s="1" t="inlineStr">
+        <is>
+          <t>A_Lo</t>
+        </is>
+      </c>
       <c r="X6" s="1" t="inlineStr">
         <is>
-          <t>A_LL Delay (sec)</t>
-        </is>
-      </c>
-      <c r="Y6" s="1" t="inlineStr"/>
+          <t>A_Lo Delay (sec)</t>
+        </is>
+      </c>
+      <c r="Y6" s="1" t="inlineStr">
+        <is>
+          <t>A_Hi</t>
+        </is>
+      </c>
       <c r="Z6" s="1" t="inlineStr">
         <is>
-          <t>A_LL Delay (sec)</t>
+          <t>A_Hi Delay (sec)</t>
         </is>
       </c>
       <c r="AA6" s="1" t="inlineStr">

</xml_diff>